<commit_message>
docs(ip-plan): IP address plan (md + xlsx + customer copy) and equipment-list update
Pre-existing working-tree artifacts from the 2026-06-05 IP-plan session,
committed so the view-modes merge starts from a clean tree.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MCCCD_AA140_Equipment_List.xlsx
+++ b/MCCCD_AA140_Equipment_List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scale\CascadeProjects\Archon-Tests\MCCCD Razzle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7FB5500-B958-4B86-9548-BD033735DB74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{828A3291-FCED-4E4E-B07B-FCC3924EC995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="128">
   <si>
     <t>MCCCD Conferencing POC (AA140 + 2 Satellite Rooms)</t>
   </si>
@@ -419,6 +419,9 @@
   </si>
   <si>
     <t>Total PO Amount: $51,961.67 (hardware + services + tax)</t>
+  </si>
+  <si>
+    <t>Arrived</t>
   </si>
 </sst>
 </file>
@@ -523,7 +526,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -561,19 +564,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -612,6 +619,16 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -888,870 +905,870 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="4" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>2</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="8">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="7" t="s">
+      <c r="D6" s="5">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="6">
-        <v>1</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="5" t="s">
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="8">
-        <v>1</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="7" t="s">
+      <c r="D8" s="5">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>2</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="5">
         <v>3</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="7" t="s">
+      <c r="E10" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>5</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="5" t="s">
+      <c r="E11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="8">
-        <v>1</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="7" t="s">
+      <c r="D12" s="5">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="6">
-        <v>1</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="5" t="s">
+      <c r="D13" s="3">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="7" t="s">
+      <c r="A14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="8">
-        <v>1</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="7" t="s">
+      <c r="D14" s="5">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="6">
-        <v>1</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="5" t="s">
+      <c r="D15" s="3">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="7" t="s">
+      <c r="A16" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="8">
-        <v>1</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="7" t="s">
+      <c r="D16" s="5">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="5" t="s">
+      <c r="A17" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D17" s="6">
-        <v>1</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="5" t="s">
+      <c r="D17" s="3">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="7" t="s">
+      <c r="A18" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="8">
-        <v>1</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" s="7" t="s">
+      <c r="D18" s="5">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="5" t="s">
+      <c r="A19" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="6">
-        <v>1</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="5" t="s">
+      <c r="D19" s="3">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="8">
-        <v>1</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="7" t="s">
+      <c r="D20" s="5">
+        <v>1</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="3">
         <v>2</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="5" t="s">
+      <c r="E21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="5">
         <v>9</v>
       </c>
-      <c r="E22" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="7" t="s">
+      <c r="E22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="5" t="s">
+      <c r="A23" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D23" s="6">
-        <v>1</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="5" t="s">
+      <c r="D23" s="3">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="8">
-        <v>1</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="7" t="s">
+      <c r="D24" s="5">
+        <v>1</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="3">
         <v>2</v>
       </c>
-      <c r="E25" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F25" s="5" t="s">
+      <c r="E25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="8">
-        <v>1</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="7" t="s">
+      <c r="D26" s="5">
+        <v>1</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="3">
         <v>2</v>
       </c>
-      <c r="E27" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F27" s="5" t="s">
+      <c r="E27" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D28" s="8">
+      <c r="D28" s="5">
         <v>4</v>
       </c>
-      <c r="E28" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F28" s="7" t="s">
+      <c r="E28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D29" s="6">
-        <v>1</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F29" s="5" t="s">
+      <c r="D29" s="3">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B30" s="7" t="s">
+      <c r="A30" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="D30" s="8">
-        <v>1</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" s="7" t="s">
+      <c r="D30" s="5">
+        <v>1</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B31" s="5" t="s">
+      <c r="A31" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D31" s="6">
-        <v>1</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F31" s="5" t="s">
+      <c r="D31" s="3">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B32" s="7" t="s">
+      <c r="A32" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D32" s="8">
-        <v>1</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="7" t="s">
+      <c r="D32" s="5">
+        <v>1</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="4" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B33" s="5" t="s">
+      <c r="A33" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D33" s="6">
-        <v>1</v>
-      </c>
-      <c r="E33" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F33" s="5" t="s">
+      <c r="D33" s="3">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D34" s="8">
-        <v>1</v>
-      </c>
-      <c r="E34" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="7" t="s">
+      <c r="D34" s="5">
+        <v>1</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="4" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D35" s="3">
         <v>14</v>
       </c>
-      <c r="E35" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F35" s="5" t="s">
+      <c r="E35" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D36" s="8">
-        <v>1</v>
-      </c>
-      <c r="E36" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F36" s="7" t="s">
+      <c r="D36" s="5">
+        <v>1</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="4" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B37" s="5" t="s">
+      <c r="A37" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D37" s="6">
+      <c r="D37" s="3">
         <v>2</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E37" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F37" s="5" t="s">
+      <c r="F37" s="2" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B38" s="7" t="s">
+      <c r="A38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D38" s="8">
+      <c r="D38" s="5">
         <v>2</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="E38" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F38" s="7" t="s">
+      <c r="F38" s="4" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B39" s="5" t="s">
+      <c r="A39" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D39" s="6">
+      <c r="D39" s="3">
         <v>2</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="E39" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F39" s="5" t="s">
+      <c r="F39" s="2" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B40" s="7" t="s">
+      <c r="A40" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D40" s="8">
+      <c r="D40" s="5">
         <v>2</v>
       </c>
-      <c r="E40" s="7" t="s">
+      <c r="E40" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F40" s="7" t="s">
+      <c r="F40" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B41" s="5" t="s">
+      <c r="A41" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D41" s="6">
+      <c r="D41" s="3">
         <v>2</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E41" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F41" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B42" s="7" t="s">
+      <c r="A42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B42" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D42" s="8">
+      <c r="D42" s="5">
         <v>2</v>
       </c>
-      <c r="E42" s="7" t="s">
+      <c r="E42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F42" s="7" t="s">
+      <c r="F42" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B43" s="5" t="s">
+      <c r="A43" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C43" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D43" s="6">
+      <c r="D43" s="3">
         <v>4</v>
       </c>
-      <c r="E43" s="5" t="s">
+      <c r="E43" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F43" s="5" t="s">
+      <c r="F43" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A44" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B44" s="7" t="s">
+      <c r="A44" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C44" s="7" t="s">
+      <c r="C44" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D44" s="8">
+      <c r="D44" s="5">
         <v>2</v>
       </c>
-      <c r="E44" s="7" t="s">
+      <c r="E44" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F44" s="7" t="s">
+      <c r="F44" s="4" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D45" s="6">
+      <c r="D45" s="3">
         <v>6</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="E45" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F45" s="5" t="s">
+      <c r="F45" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D46" s="12">
+      <c r="D46" s="9">
         <f>SUM(D5:D45)</f>
         <v>91</v>
       </c>
@@ -1768,7 +1785,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1777,553 +1794,608 @@
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="4" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+    </row>
+    <row r="4" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="5" t="s">
+    <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>3</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="14" t="s">
+      <c r="G5" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="12">
         <v>5</v>
       </c>
-      <c r="E6" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="14" t="s">
+      <c r="E6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="G6" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="6">
-        <v>1</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="5" t="s">
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="14" t="s">
+      <c r="G7" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="15">
-        <v>1</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="14" t="s">
+      <c r="D8" s="12">
+        <v>1</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="G8" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="6">
-        <v>1</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="5" t="s">
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="14" t="s">
+      <c r="G9" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="15">
-        <v>1</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="14" t="s">
+      <c r="D10" s="12">
+        <v>1</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="11" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="5" t="s">
+      <c r="G10" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="6">
-        <v>1</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="5" t="s">
+      <c r="D11" s="3">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="14" t="s">
+      <c r="G11" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="15">
-        <v>1</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="14" t="s">
+      <c r="D12" s="12">
+        <v>1</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="11" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="5" t="s">
+      <c r="G12" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="6">
-        <v>1</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="5" t="s">
+      <c r="D13" s="3">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="14" t="s">
+      <c r="G13" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="15">
-        <v>1</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="14" t="s">
+      <c r="D14" s="12">
+        <v>1</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="5" t="s">
+    <row r="15" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="3">
         <v>2</v>
       </c>
-      <c r="E15" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="5" t="s">
+      <c r="E15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="14" t="s">
+    <row r="16" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="12">
         <v>9</v>
       </c>
-      <c r="E16" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="14" t="s">
+      <c r="E16" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="11" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="5" t="s">
+    <row r="17" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="6">
-        <v>1</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="5" t="s">
+      <c r="D17" s="3">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="14" t="s">
+    <row r="18" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D18" s="15">
-        <v>1</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" s="14" t="s">
+      <c r="D18" s="12">
+        <v>1</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="11" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="5" t="s">
+      <c r="G18" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="6">
-        <v>1</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="5" t="s">
+      <c r="D19" s="3">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" s="14" t="s">
+      <c r="G19" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="D20" s="15">
-        <v>1</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="14" t="s">
+      <c r="D20" s="12">
+        <v>1</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="11" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="5" t="s">
+      <c r="G20" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="6">
-        <v>1</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="5" t="s">
+      <c r="D21" s="3">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" s="14" t="s">
+      <c r="G21" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C22" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="12">
         <v>2</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="E22" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F22" s="11" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="5" t="s">
+      <c r="G22" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="3">
         <v>2</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" s="14" t="s">
+      <c r="G23" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="C24" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="12">
         <v>2</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="E24" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="F24" s="11" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B25" s="5" t="s">
+      <c r="G24" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="3">
         <v>2</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="14" t="s">
+      <c r="G25" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="C26" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="12">
         <v>2</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="F26" s="11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" s="5" t="s">
+      <c r="G26" s="18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="3">
         <v>2</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E27" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="F27" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="14" t="s">
+    <row r="28" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="12">
         <v>4</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="E28" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="F28" s="11" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" s="5" t="s">
+    <row r="29" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="3">
         <v>2</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F29" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C30" s="11" t="s">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C30" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="9">
         <f>SUM(D5:D29)</f>
         <v>50</v>
       </c>
@@ -2347,105 +2419,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17"/>
+      <c r="A2" s="14"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="14" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="14" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="14" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
+      <c r="A6" s="14"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="14" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
+      <c r="A8" s="14"/>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="14" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
+      <c r="A10" s="14"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="14" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
+      <c r="A12" s="14"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="14" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="14" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="14" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="14" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="14" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="14" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="14" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="14" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="14" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17"/>
+      <c r="A22" s="14"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="14" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>